<commit_message>
HOLD: Excel-safe template ranges, 30d churn, Canceled spelling
Bound Dashboard formulas to A2:A10000-style ranges (Excel rejects
Sheets A2:A open ends). CHURN · 30D uses the Canceled date column
over a trailing 30 days. Rename Cancelled → Canceled to match status
spelling. Reject open-ended ranges in every xlsx formula via test.

Co-authored-by: Gatlin Farrington <gatlinfarrington@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/revenuesheet-template.xlsx
+++ b/public/revenuesheet-template.xlsx
@@ -464,167 +464,7 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B1:N14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Revenue dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Blank template · formulas stay at zero until rows are added</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>MRR</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>NET REVENUE · 30D</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>ACTIVE SUBSCRIPTIONS</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>CHURN · 30D</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="4">
-        <f>SUMIF(Subscriptions!H:H,"active",Subscriptions!G:G)</f>
-        <v/>
-      </c>
-      <c r="F5" s="4">
-        <f>SUMIF(Orders!H:H,"paid",Orders!G:G)-SUMIF(Refunds!G:G,"succeeded",Refunds!F:F)-SUMIF(Refunds!G:G,"paid",Refunds!F:F)</f>
-        <v/>
-      </c>
-      <c r="J5" s="5">
-        <f>COUNTIF(Subscriptions!H:H,"active")</f>
-        <v/>
-      </c>
-      <c r="N5" s="6">
-        <f>IFERROR(COUNTIF(Subscriptions!H:H,"canceled")/(COUNTIF(Subscriptions!H:H,"active")+COUNTIF(Subscriptions!H:H,"canceled")),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Active subscriptions only</t>
-        </is>
-      </c>
-      <c r="F6" s="2">
-        <f>COUNTA(Orders!A2:A)&amp;" orders (all time)"</f>
-        <v/>
-      </c>
-      <c r="J6" s="2">
-        <f>COUNTIF(Subscriptions!H:H,"past_due")&amp;" past due"</f>
-        <v/>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>Uses Status column; 0 when empty</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Orders</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Customers</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>Refunds</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="5">
-        <f>COUNTA(Orders!A2:A)</f>
-        <v/>
-      </c>
-      <c r="F9" s="5">
-        <f>COUNTA(Customers!A2:A)</f>
-        <v/>
-      </c>
-      <c r="J9" s="5">
-        <f>COUNTA(Refunds!A2:A)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>row count</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>row count</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>row count</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>How to use</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Keep these tab names and header rows. The add-on writes into the same columns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>This file is a blank layout preview — not an installable add-on.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
+<file path=xl/worksheets/sheet1.xml><worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"><sheetPr><outlinePr summaryBelow="1" summaryRight="1" /><pageSetUpPr /></sheetPr><dimension ref="B1:N14" /><sheetFormatPr baseColWidth="8" defaultRowHeight="15" /><cols><col width="28" customWidth="1" min="2" max="2" /><col width="28" customWidth="1" min="6" max="6" /><col width="24" customWidth="1" min="10" max="10" /><col width="18" customWidth="1" min="14" max="14" /></cols><sheetData><row r="1"><c r="B1" s="1" t="inlineStr"><is><t>Revenue dashboard</t></is></c></row><row r="2"><c r="B2" s="2" t="inlineStr"><is><t>Blank template · formulas stay at zero until rows are added</t></is></c></row><row r="4"><c r="B4" s="3" t="inlineStr"><is><t>MRR</t></is></c><c r="F4" s="3" t="inlineStr"><is><t>NET REVENUE · 30D</t></is></c><c r="J4" s="3" t="inlineStr"><is><t>ACTIVE SUBSCRIPTIONS</t></is></c><c r="N4" s="3" t="inlineStr"><is><t>CHURN · 30D</t></is></c></row><row r="5"><c r="B5" s="4"><f>SUMIF(Subscriptions!H2:H10000,"active",Subscriptions!G2:G10000)</f><v /></c><c r="F5" s="4"><f>SUMIF(Orders!H2:H10000,"paid",Orders!G2:G10000)-SUMIF(Refunds!G2:G10000,"succeeded",Refunds!F2:F10000)-SUMIF(Refunds!G2:G10000,"paid",Refunds!F2:F10000)</f><v /></c><c r="J5" s="5"><f>COUNTIF(Subscriptions!H2:H10000,"active")</f><v /></c><c r="N5" s="6"><f>IFERROR(COUNTIFS(Subscriptions!I2:I10000,">="&amp;TODAY()-30,Subscriptions!I2:I10000,"<>")/(COUNTIF(Subscriptions!H2:H10000,"active")+COUNTIFS(Subscriptions!I2:I10000,">="&amp;TODAY()-30,Subscriptions!I2:I10000,"<>")),0)</f><v /></c></row><row r="6"><c r="B6" s="2" t="inlineStr"><is><t>Active subscriptions only</t></is></c><c r="F6" s="2"><f>COUNTA(Orders!A2:A10000)&amp;" orders (all time)"</f><v /></c><c r="J6" s="2"><f>COUNTIF(Subscriptions!H2:H10000,"past_due")&amp;" past due"</f><v /></c><c r="N6" s="2" t="inlineStr"><is><t>Canceled in last 30 days ÷ (active + canceled in window)</t></is></c></row><row r="8"><c r="B8" s="3" t="inlineStr"><is><t>Orders</t></is></c><c r="F8" s="3" t="inlineStr"><is><t>Customers</t></is></c><c r="J8" s="3" t="inlineStr"><is><t>Refunds</t></is></c></row><row r="9"><c r="B9" s="5"><f>COUNTA(Orders!A2:A10000)</f><v /></c><c r="F9" s="5"><f>COUNTA(Customers!A2:A10000)</f><v /></c><c r="J9" s="5"><f>COUNTA(Refunds!A2:A10000)</f><v /></c></row><row r="10"><c r="B10" s="2" t="inlineStr"><is><t>row count</t></is></c><c r="F10" s="2" t="inlineStr"><is><t>row count</t></is></c><c r="J10" s="2" t="inlineStr"><is><t>row count</t></is></c></row><row r="12"><c r="B12" s="3" t="inlineStr"><is><t>How to use</t></is></c></row><row r="13"><c r="B13" s="2" t="inlineStr"><is><t>Keep these tab names and header rows. The add-on writes into the same columns.</t></is></c></row><row r="14"><c r="B14" s="2" t="inlineStr"><is><t>This file is a blank layout preview — not an installable add-on.</t></is></c></row></sheetData><pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5" /></worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -765,7 +605,7 @@
       </c>
       <c r="I1" s="7" t="inlineStr">
         <is>
-          <t>Cancelled</t>
+          <t>Canceled</t>
         </is>
       </c>
       <c r="J1" s="7" t="inlineStr">

</xml_diff>

<commit_message>
HOLD: XML-escape template formulas; openpyxl + LibreOffice checks
N5 churn used raw <> which broke sheet1.xml (Excel repair / openpyxl
ParseError). Rebuild via escapeXml for every formula and string.
Strict XML + openpyxl KPI assert in CI; LibreOffice recalc when present.

Co-authored-by: Gatlin Farrington <gatlinfarrington@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/revenuesheet-template.xlsx
+++ b/public/revenuesheet-template.xlsx
@@ -464,291 +464,392 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"><sheetPr><outlinePr summaryBelow="1" summaryRight="1" /><pageSetUpPr /></sheetPr><dimension ref="B1:N14" /><sheetFormatPr baseColWidth="8" defaultRowHeight="15" /><cols><col width="28" customWidth="1" min="2" max="2" /><col width="28" customWidth="1" min="6" max="6" /><col width="24" customWidth="1" min="10" max="10" /><col width="18" customWidth="1" min="14" max="14" /></cols><sheetData><row r="1"><c r="B1" s="1" t="inlineStr"><is><t>Revenue dashboard</t></is></c></row><row r="2"><c r="B2" s="2" t="inlineStr"><is><t>Blank template · formulas stay at zero until rows are added</t></is></c></row><row r="4"><c r="B4" s="3" t="inlineStr"><is><t>MRR</t></is></c><c r="F4" s="3" t="inlineStr"><is><t>NET REVENUE · 30D</t></is></c><c r="J4" s="3" t="inlineStr"><is><t>ACTIVE SUBSCRIPTIONS</t></is></c><c r="N4" s="3" t="inlineStr"><is><t>CHURN · 30D</t></is></c></row><row r="5"><c r="B5" s="4"><f>SUMIF(Subscriptions!H2:H10000,"active",Subscriptions!G2:G10000)</f><v /></c><c r="F5" s="4"><f>SUMIF(Orders!H2:H10000,"paid",Orders!G2:G10000)-SUMIF(Refunds!G2:G10000,"succeeded",Refunds!F2:F10000)-SUMIF(Refunds!G2:G10000,"paid",Refunds!F2:F10000)</f><v /></c><c r="J5" s="5"><f>COUNTIF(Subscriptions!H2:H10000,"active")</f><v /></c><c r="N5" s="6"><f>IFERROR(COUNTIFS(Subscriptions!I2:I10000,">="&amp;TODAY()-30,Subscriptions!I2:I10000,"<>")/(COUNTIF(Subscriptions!H2:H10000,"active")+COUNTIFS(Subscriptions!I2:I10000,">="&amp;TODAY()-30,Subscriptions!I2:I10000,"<>")),0)</f><v /></c></row><row r="6"><c r="B6" s="2" t="inlineStr"><is><t>Active subscriptions only</t></is></c><c r="F6" s="2"><f>COUNTA(Orders!A2:A10000)&amp;" orders (all time)"</f><v /></c><c r="J6" s="2"><f>COUNTIF(Subscriptions!H2:H10000,"past_due")&amp;" past due"</f><v /></c><c r="N6" s="2" t="inlineStr"><is><t>Canceled in last 30 days ÷ (active + canceled in window)</t></is></c></row><row r="8"><c r="B8" s="3" t="inlineStr"><is><t>Orders</t></is></c><c r="F8" s="3" t="inlineStr"><is><t>Customers</t></is></c><c r="J8" s="3" t="inlineStr"><is><t>Refunds</t></is></c></row><row r="9"><c r="B9" s="5"><f>COUNTA(Orders!A2:A10000)</f><v /></c><c r="F9" s="5"><f>COUNTA(Customers!A2:A10000)</f><v /></c><c r="J9" s="5"><f>COUNTA(Refunds!A2:A10000)</f><v /></c></row><row r="10"><c r="B10" s="2" t="inlineStr"><is><t>row count</t></is></c><c r="F10" s="2" t="inlineStr"><is><t>row count</t></is></c><c r="J10" s="2" t="inlineStr"><is><t>row count</t></is></c></row><row r="12"><c r="B12" s="3" t="inlineStr"><is><t>How to use</t></is></c></row><row r="13"><c r="B13" s="2" t="inlineStr"><is><t>Keep these tab names and header rows. The add-on writes into the same columns.</t></is></c></row><row r="14"><c r="B14" s="2" t="inlineStr"><is><t>This file is a blank layout preview — not an installable add-on.</t></is></c></row></sheetData><pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5" /></worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="B1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Revenue dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Blank template · formulas stay at zero until rows are added</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>MRR</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>NET REVENUE · 30D</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE SUBSCRIPTIONS</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>CHURN · 30D</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="4">
+        <f>SUMIF(Subscriptions!H2:H10000,"active",Subscriptions!G2:G10000)</f>
+        <v/>
+      </c>
+      <c r="F5" s="4">
+        <f>SUMIF(Orders!H2:H10000,"paid",Orders!G2:G10000)-SUMIF(Refunds!G2:G10000,"succeeded",Refunds!F2:F10000)-SUMIF(Refunds!G2:G10000,"paid",Refunds!F2:F10000)</f>
+        <v/>
+      </c>
+      <c r="J5" s="5">
+        <f>COUNTIF(Subscriptions!H2:H10000,"active")</f>
+        <v/>
+      </c>
+      <c r="N5" s="6">
+        <f>IFERROR(COUNTIFS(Subscriptions!I2:I10000,"&gt;="&amp;TODAY()-30,Subscriptions!I2:I10000,"&lt;&gt;")/(COUNTIF(Subscriptions!H2:H10000,"active")+COUNTIFS(Subscriptions!I2:I10000,"&gt;="&amp;TODAY()-30,Subscriptions!I2:I10000,"&lt;&gt;")),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Active subscriptions only</t>
+        </is>
+      </c>
+      <c r="F6" s="2">
+        <f>COUNTA(Orders!A2:A10000)&amp;" orders (all time)"</f>
+        <v/>
+      </c>
+      <c r="J6" s="2">
+        <f>COUNTIF(Subscriptions!H2:H10000,"past_due")&amp;" past due"</f>
+        <v/>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Canceled in last 30 days ÷ (active + canceled in window)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Customers</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Refunds</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="5">
+        <f>COUNTA(Orders!A2:A10000)</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>COUNTA(Customers!A2:A10000)</f>
+        <v/>
+      </c>
+      <c r="J9" s="5">
+        <f>COUNTA(Refunds!A2:A10000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>row count</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>row count</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>row count</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>How to use</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Keep these tab names and header rows. The add-on writes into the same columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>This file is a blank layout preview — not an installable add-on.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr/>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Order ID</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Created</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Customer email</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Amount (USD)</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+  <sheetPr/>
   <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Subscription ID</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Created</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Customer email</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>MRR (USD)</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Canceled</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Interval</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+  <sheetPr/>
   <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Customer ID</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Created</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+  <sheetPr/>
   <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Refund ID</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Created</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Order ID</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Amount (USD)</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>